<commit_message>
XC9500-IO: routed board, add EXTERNAL MCP11/12 SPI header P21
Source: S100 XC9500 Ver1/backups/29-07-2015 1801. First routed layout (Specctra session imported).
</commit_message>
<xml_diff>
--- a/XC9500-IO/XC9500v1.xlsx
+++ b/XC9500-IO/XC9500v1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="87">
   <si>
     <t>0.1 uF</t>
   </si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>663-2195</t>
+  </si>
+  <si>
+    <t>712-2576</t>
   </si>
 </sst>
 </file>
@@ -1281,7 +1284,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1292,7 +1295,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1303,7 +1306,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -1314,7 +1317,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -1325,7 +1328,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1336,7 +1339,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -1347,7 +1350,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1358,7 +1361,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1369,7 +1372,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1380,7 +1383,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:13">
       <c r="A26">
         <v>50</v>
       </c>
@@ -1391,7 +1394,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:13">
       <c r="A27">
         <v>100</v>
       </c>
@@ -1402,7 +1405,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:13">
       <c r="A28">
         <v>330</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -1424,7 +1427,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -1435,7 +1438,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1446,7 +1449,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
         <v>55</v>
       </c>
@@ -1455,6 +1458,9 @@
       </c>
       <c r="C32" t="s">
         <v>56</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:13">

</xml_diff>